<commit_message>
fixed a date in SLS turbidity
</commit_message>
<xml_diff>
--- a/data_raw/smelt/SLS catch update1.26.26.xlsx
+++ b/data_raw/smelt/SLS catch update1.26.26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/geasterbrook_usbr_gov/Documents/My Projects/SMT/Assessment/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD71539D-E068-4AE0-8495-D52A1D2F9104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{CD71539D-E068-4AE0-8495-D52A1D2F9104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18E3D5DC-1F82-4510-ADBB-4A74BDFAED93}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{E318DA66-929E-4160-AE8F-A3EAE62CC340}"/>
   </bookViews>
@@ -742,7 +742,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1007,6 +1007,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9028,7 +9030,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47866F3D-7537-4F6F-BFFA-DC500CC10CD5}">
-  <dimension ref="A1:N64"/>
+  <dimension ref="A1:Q64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -10760,7 +10762,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="75">
         <v>2026</v>
       </c>
@@ -10804,7 +10806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="75">
         <v>2026</v>
       </c>
@@ -10837,8 +10839,10 @@
       <c r="L50" s="3"/>
       <c r="M50" s="30"/>
       <c r="N50" s="33"/>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P50" s="98"/>
+      <c r="Q50" s="99"/>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="53">
         <v>2026</v>
       </c>
@@ -10872,7 +10876,7 @@
       <c r="M51" s="29"/>
       <c r="N51" s="32"/>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" s="53">
         <v>2026</v>
       </c>
@@ -10906,7 +10910,7 @@
       <c r="M52" s="29"/>
       <c r="N52" s="32"/>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="53">
         <v>2026</v>
       </c>
@@ -10940,7 +10944,7 @@
       <c r="M53" s="29"/>
       <c r="N53" s="32"/>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" s="53">
         <v>2026</v>
       </c>
@@ -10974,7 +10978,7 @@
       <c r="M54" s="29"/>
       <c r="N54" s="32"/>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="53">
         <v>2026</v>
       </c>
@@ -11008,7 +11012,7 @@
       <c r="M55" s="29"/>
       <c r="N55" s="32"/>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" s="53">
         <v>2026</v>
       </c>
@@ -11042,7 +11046,7 @@
       <c r="M56" s="29"/>
       <c r="N56" s="32"/>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="53">
         <v>2026</v>
       </c>
@@ -11076,7 +11080,7 @@
       <c r="M57" s="29"/>
       <c r="N57" s="32"/>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="53">
         <v>2026</v>
       </c>
@@ -11110,7 +11114,7 @@
       <c r="M58" s="29"/>
       <c r="N58" s="32"/>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="53">
         <v>2026</v>
       </c>
@@ -11144,7 +11148,7 @@
       <c r="M59" s="29"/>
       <c r="N59" s="32"/>
     </row>
-    <row r="60" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="76">
         <v>2026</v>
       </c>
@@ -11178,7 +11182,7 @@
       <c r="M60" s="73"/>
       <c r="N60" s="74"/>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="80" t="s">
         <v>39</v>
       </c>
@@ -11196,7 +11200,7 @@
       <c r="M61" s="43"/>
       <c r="N61" s="6"/>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="80" t="s">
         <v>40</v>
       </c>
@@ -11214,7 +11218,7 @@
       <c r="M62" s="44"/>
       <c r="N62" s="28"/>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="80" t="s">
         <v>41</v>
       </c>
@@ -11232,7 +11236,7 @@
       <c r="M63" s="60"/>
       <c r="N63" s="36"/>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="83" t="s">
         <v>42</v>
       </c>
@@ -11299,4 +11303,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" enabled="0" method="" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>